<commit_message>
add asa concept note approval
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_eap.xlsx
+++ b/inst/extdata/wb_projects_gov_eap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -33,6 +33,12 @@
     <t xml:space="preserve">proj_approval_fy</t>
   </si>
   <si>
+    <t xml:space="preserve">asa_cn_approval_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">task_type</t>
+  </si>
+  <si>
     <t xml:space="preserve">proj_url</t>
   </si>
   <si>
@@ -147,6 +153,9 @@
     <t xml:space="preserve">Democratic Republic of Timor-Leste</t>
   </si>
   <si>
+    <t xml:space="preserve">Advisory</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://opswork.worldbank.org/home/P501950</t>
   </si>
   <si>
@@ -166,6 +175,9 @@
   </si>
   <si>
     <t xml:space="preserve">Kingdom of Cambodia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytical</t>
   </si>
   <si>
     <t xml:space="preserve">https://opswork.worldbank.org/home/P513817</t>
@@ -199,7 +211,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="yyyy/mm/dd hh:mm:ss"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -234,8 +248,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -535,238 +550,252 @@
     <col min="4" max="4" width="21.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="37.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="42.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="17.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="18.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="7.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="29.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="17.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="9.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="9.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="42.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="17.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="18.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="7.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="29.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="18.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="16.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="8.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="9.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="16.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="P2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" s="1" t="s">
+      <c r="M2" s="2" t="s">
         <v>29</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="O3" s="2"/>
+      <c r="P3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="A4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="1" t="n">
+      <c r="C4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="1" t="s">
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="L4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" s="1" t="s">
+      <c r="M4" s="2" t="s">
         <v>29</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -786,272 +815,296 @@
     <col min="4" max="4" width="21.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="37.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="42.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="40.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="18.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="7.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="24.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="17.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="9.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="10.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="42.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="40.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="18.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="7.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="24.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
     <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="18.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="16.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="8.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="9.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="16.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="1" t="n">
+      <c r="C2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" s="1" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>29</v>
+      <c r="I2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>29</v>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" s="1" t="n">
+      <c r="F4" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>29</v>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="1" t="n">
+      <c r="A5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>29</v>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>